<commit_message>
Included all data, done residuals, and excluded the outliers
</commit_message>
<xml_diff>
--- a/Cell survival results/2026_3_11/Multiplicity X-rays 11-3.xlsx
+++ b/Cell survival results/2026_3_11/Multiplicity X-rays 11-3.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29910"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="209" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D164BFA-2549-40C2-A9A8-53F37CC5EAD5}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhaan\Documents\#Master Degree\Thesis\Thesis_project\Cell survival results\2026_3_11\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8847EFA7-88C5-40FF-9A7E-F30A4909A393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -79,7 +84,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -454,9 +459,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -473,7 +478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -491,7 +496,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -509,7 +514,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -527,7 +532,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -545,7 +550,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -563,7 +568,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -581,7 +586,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -599,7 +604,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -617,7 +622,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -635,7 +640,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -653,7 +658,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
@@ -671,7 +676,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -689,7 +694,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>

</xml_diff>